<commit_message>
Encore une fois 25c734ba0d932d34c2f691cfdca28a1efc103ae0
</commit_message>
<xml_diff>
--- a/AnalysePharma/ig/StructureDefinition-fr-inpatient-pharmaceutical-analysis-result.xlsx
+++ b/AnalysePharma/ig/StructureDefinition-fr-inpatient-pharmaceutical-analysis-result.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4041" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4041" uniqueCount="519">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-16T16:30:02+00:00</t>
+    <t>2026-02-16T17:09:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1351,7 +1351,7 @@
     <t>Task.input.value[x]</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/medication/StructureDefinition/fr-inpatient-medicationrequest)
 </t>
   </si>
   <si>
@@ -1619,6 +1619,10 @@
   </si>
   <si>
     <t>Task.output:suggestion.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/medication/StructureDefinition/fr-inpatient-pharmaceutical-intervention-suggestion)
+</t>
   </si>
 </sst>
 </file>
@@ -14563,7 +14567,7 @@
         <v>77</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>429</v>
+        <v>518</v>
       </c>
       <c r="L111" t="s" s="2">
         <v>448</v>

</xml_diff>

<commit_message>
fix forbidden letter 38e3df48fe534beb23b5b62e8a8dcf536426c766
</commit_message>
<xml_diff>
--- a/AnalysePharma/ig/StructureDefinition-fr-inpatient-pharmaceutical-analysis-result.xlsx
+++ b/AnalysePharma/ig/StructureDefinition-fr-inpatient-pharmaceutical-analysis-result.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$121</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4041" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4402" uniqueCount="531">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-17T10:22:56+00:00</t>
+    <t>2026-04-14T15:08:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -647,7 +647,10 @@
     <t>There's often a need to track substates of a task - this is often variable by specific workflow implementation.</t>
   </si>
   <si>
-    <t>The domain-specific business-contextual sub-state of the task.  For example: "Blood drawn", "IV inserted", "Awaiting physician signature", etc.</t>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/medication/ValueSet/fr-pharmaceutical-intervention-devenir-code-value-set</t>
   </si>
   <si>
     <t>.inboundRelationship[typeCode=SUBJ].source[classCode=OBS, moodCode=EVN, code="business status"]</t>
@@ -936,9 +939,6 @@
     <t>Use to distinguish tasks on different activity queues.</t>
   </si>
   <si>
-    <t>extensible</t>
-  </si>
-  <si>
     <t>https://hl7.fr/ig/fhir/medication/ValueSet/fr-pharmaceutical-analysis-perfomer-type-value-set</t>
   </si>
   <si>
@@ -1623,6 +1623,42 @@
   <si>
     <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/medication/StructureDefinition/fr-inpatient-pharmaceutical-intervention-suggestion)
 </t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated</t>
+  </si>
+  <si>
+    <t>suggestionUpdated</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.id</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.extension</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.modifierExtension</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.type</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.type.id</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.type.extension</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.type.coding</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.type.text</t>
+  </si>
+  <si>
+    <t>proposition modifiée</t>
+  </si>
+  <si>
+    <t>Task.output:suggestionUpdated.value[x]</t>
   </si>
 </sst>
 </file>
@@ -1939,12 +1975,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN111"/>
+  <dimension ref="A1:AN121"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="34.11328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="40.8046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="27.80078125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="16.19140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -4102,13 +4138,11 @@
         <v>77</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="Y19" t="s" s="2">
         <v>203</v>
       </c>
+      <c r="Y19" s="2"/>
       <c r="Z19" t="s" s="2">
-        <v>77</v>
+        <v>204</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>77</v>
@@ -4144,7 +4178,7 @@
         <v>77</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>77</v>
@@ -4155,10 +4189,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4184,13 +4218,13 @@
         <v>107</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -4201,7 +4235,7 @@
         <v>77</v>
       </c>
       <c r="S20" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="T20" t="s" s="2">
         <v>77</v>
@@ -4219,10 +4253,10 @@
         <v>186</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>77</v>
@@ -4240,7 +4274,7 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>87</v>
@@ -4255,13 +4289,13 @@
         <v>99</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AN20" t="s" s="2">
         <v>77</v>
@@ -4269,10 +4303,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4298,20 +4332,20 @@
         <v>107</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>77</v>
       </c>
       <c r="Q21" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="R21" t="s" s="2">
         <v>77</v>
@@ -4335,10 +4369,10 @@
         <v>186</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>77</v>
@@ -4356,7 +4390,7 @@
         <v>77</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
@@ -4371,13 +4405,13 @@
         <v>99</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AN21" t="s" s="2">
         <v>77</v>
@@ -4385,10 +4419,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4414,13 +4448,13 @@
         <v>192</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -4449,10 +4483,10 @@
         <v>196</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>77</v>
@@ -4470,7 +4504,7 @@
         <v>77</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
@@ -4485,13 +4519,13 @@
         <v>99</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AN22" t="s" s="2">
         <v>77</v>
@@ -4499,10 +4533,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4525,13 +4559,13 @@
         <v>88</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -4582,7 +4616,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4600,7 +4634,7 @@
         <v>77</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="AM23" t="s" s="2">
         <v>77</v>
@@ -4611,10 +4645,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4640,16 +4674,16 @@
         <v>163</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>77</v>
@@ -4698,7 +4732,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4716,10 +4750,10 @@
         <v>77</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>77</v>
@@ -4727,14 +4761,14 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
@@ -4756,14 +4790,14 @@
         <v>163</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>77</v>
@@ -4812,7 +4846,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4827,13 +4861,13 @@
         <v>99</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>77</v>
@@ -4841,10 +4875,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4867,17 +4901,17 @@
         <v>88</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>77</v>
@@ -4926,7 +4960,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4941,13 +4975,13 @@
         <v>99</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>77</v>
@@ -4955,10 +4989,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4981,13 +5015,13 @@
         <v>88</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -5038,7 +5072,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -5053,13 +5087,13 @@
         <v>99</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>77</v>
@@ -5067,14 +5101,14 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
@@ -5093,17 +5127,17 @@
         <v>77</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>77</v>
@@ -5152,7 +5186,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -5161,19 +5195,19 @@
         <v>87</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AJ28" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>77</v>
@@ -5181,14 +5215,14 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -5207,17 +5241,17 @@
         <v>88</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>77</v>
@@ -5266,7 +5300,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -5275,7 +5309,7 @@
         <v>87</v>
       </c>
       <c r="AI29" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AJ29" t="s" s="2">
         <v>99</v>
@@ -5284,7 +5318,7 @@
         <v>77</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>77</v>
@@ -5295,10 +5329,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5321,17 +5355,17 @@
         <v>88</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>77</v>
@@ -5380,7 +5414,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -5395,13 +5429,13 @@
         <v>99</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>77</v>
@@ -5409,10 +5443,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5438,14 +5472,14 @@
         <v>192</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>77</v>
@@ -5470,7 +5504,7 @@
         <v>77</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>296</v>
+        <v>203</v>
       </c>
       <c r="Y31" s="2"/>
       <c r="Z31" t="s" s="2">
@@ -5492,7 +5526,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -6457,7 +6491,7 @@
         <v>77</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L40" t="s" s="2">
         <v>360</v>
@@ -6913,7 +6947,7 @@
         <v>77</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L44" t="s" s="2">
         <v>379</v>
@@ -7255,7 +7289,7 @@
         <v>77</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L47" t="s" s="2">
         <v>360</v>
@@ -7713,7 +7747,7 @@
         <v>77</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L51" t="s" s="2">
         <v>360</v>
@@ -8055,7 +8089,7 @@
         <v>88</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L54" t="s" s="2">
         <v>420</v>
@@ -8397,7 +8431,7 @@
         <v>77</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L57" t="s" s="2">
         <v>360</v>
@@ -9083,7 +9117,7 @@
         <v>77</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L63" t="s" s="2">
         <v>360</v>
@@ -9539,7 +9573,7 @@
         <v>77</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L67" t="s" s="2">
         <v>360</v>
@@ -9881,7 +9915,7 @@
         <v>88</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L70" t="s" s="2">
         <v>420</v>
@@ -10225,7 +10259,7 @@
         <v>77</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L73" t="s" s="2">
         <v>360</v>
@@ -10681,7 +10715,7 @@
         <v>77</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L77" t="s" s="2">
         <v>360</v>
@@ -11023,7 +11057,7 @@
         <v>88</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L80" t="s" s="2">
         <v>420</v>
@@ -11139,7 +11173,7 @@
         <v>77</v>
       </c>
       <c r="K81" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L81" t="s" s="2">
         <v>448</v>
@@ -11369,7 +11403,7 @@
         <v>77</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L83" t="s" s="2">
         <v>360</v>
@@ -11825,7 +11859,7 @@
         <v>77</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L87" t="s" s="2">
         <v>360</v>
@@ -12167,7 +12201,7 @@
         <v>88</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L90" t="s" s="2">
         <v>420</v>
@@ -12318,7 +12352,7 @@
         <v>77</v>
       </c>
       <c r="X91" t="s" s="2">
-        <v>296</v>
+        <v>203</v>
       </c>
       <c r="Y91" s="2"/>
       <c r="Z91" t="s" s="2">
@@ -12511,7 +12545,7 @@
         <v>77</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L93" t="s" s="2">
         <v>360</v>
@@ -12967,7 +13001,7 @@
         <v>77</v>
       </c>
       <c r="K97" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L97" t="s" s="2">
         <v>360</v>
@@ -13309,7 +13343,7 @@
         <v>88</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L100" t="s" s="2">
         <v>420</v>
@@ -13460,7 +13494,7 @@
         <v>77</v>
       </c>
       <c r="X101" t="s" s="2">
-        <v>296</v>
+        <v>203</v>
       </c>
       <c r="Y101" s="2"/>
       <c r="Z101" t="s" s="2">
@@ -13653,7 +13687,7 @@
         <v>77</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L103" t="s" s="2">
         <v>360</v>
@@ -14109,7 +14143,7 @@
         <v>77</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L107" t="s" s="2">
         <v>360</v>
@@ -14451,7 +14485,7 @@
         <v>88</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L110" t="s" s="2">
         <v>420</v>
@@ -14653,8 +14687,1152 @@
         <v>77</v>
       </c>
     </row>
+    <row r="112" hidden="true">
+      <c r="A112" t="s" s="2">
+        <v>519</v>
+      </c>
+      <c r="B112" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="C112" t="s" s="2">
+        <v>520</v>
+      </c>
+      <c r="D112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E112" s="2"/>
+      <c r="F112" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G112" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K112" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="L112" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="M112" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="N112" s="2"/>
+      <c r="O112" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="P112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q112" s="2"/>
+      <c r="R112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF112" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="AG112" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH112" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ112" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL112" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AM112" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN112" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="113" hidden="true">
+      <c r="A113" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="B113" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="C113" s="2"/>
+      <c r="D113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E113" s="2"/>
+      <c r="F113" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G113" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K113" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="L113" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="M113" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="N113" s="2"/>
+      <c r="O113" s="2"/>
+      <c r="P113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q113" s="2"/>
+      <c r="R113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF113" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="AG113" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH113" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AK113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL113" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AM113" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN113" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="114" hidden="true">
+      <c r="A114" t="s" s="2">
+        <v>522</v>
+      </c>
+      <c r="B114" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="C114" s="2"/>
+      <c r="D114" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="E114" s="2"/>
+      <c r="F114" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G114" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K114" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L114" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="M114" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N114" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O114" s="2"/>
+      <c r="P114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q114" s="2"/>
+      <c r="R114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF114" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="AG114" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH114" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ114" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL114" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AM114" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN114" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="115" hidden="true">
+      <c r="A115" t="s" s="2">
+        <v>523</v>
+      </c>
+      <c r="B115" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="C115" s="2"/>
+      <c r="D115" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="E115" s="2"/>
+      <c r="F115" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G115" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I115" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="J115" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K115" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L115" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="M115" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="N115" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O115" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="P115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q115" s="2"/>
+      <c r="R115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF115" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AG115" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH115" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ115" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL115" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="AM115" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN115" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="116" hidden="true">
+      <c r="A116" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="B116" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="C116" s="2"/>
+      <c r="D116" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="E116" s="2"/>
+      <c r="F116" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G116" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K116" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="L116" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="M116" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="N116" s="2"/>
+      <c r="O116" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="P116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q116" s="2"/>
+      <c r="R116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X116" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="Y116" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="Z116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF116" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="AG116" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH116" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ116" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL116" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AM116" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN116" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="117" hidden="true">
+      <c r="A117" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="B117" t="s" s="2">
+        <v>458</v>
+      </c>
+      <c r="C117" s="2"/>
+      <c r="D117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E117" s="2"/>
+      <c r="F117" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G117" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K117" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="L117" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="M117" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="N117" s="2"/>
+      <c r="O117" s="2"/>
+      <c r="P117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q117" s="2"/>
+      <c r="R117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF117" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="AG117" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH117" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AK117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL117" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AM117" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN117" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="118" hidden="true">
+      <c r="A118" t="s" s="2">
+        <v>526</v>
+      </c>
+      <c r="B118" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="C118" s="2"/>
+      <c r="D118" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="E118" s="2"/>
+      <c r="F118" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G118" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K118" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L118" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="M118" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N118" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O118" s="2"/>
+      <c r="P118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q118" s="2"/>
+      <c r="R118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB118" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="AC118" t="s" s="2">
+        <v>408</v>
+      </c>
+      <c r="AD118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE118" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="AF118" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="AG118" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH118" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ118" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL118" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AM118" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN118" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="119" hidden="true">
+      <c r="A119" t="s" s="2">
+        <v>527</v>
+      </c>
+      <c r="B119" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="C119" s="2"/>
+      <c r="D119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E119" s="2"/>
+      <c r="F119" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G119" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J119" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K119" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="L119" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="M119" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="N119" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="O119" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="P119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q119" s="2"/>
+      <c r="R119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF119" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="AG119" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH119" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ119" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL119" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="AM119" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN119" t="s" s="2">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="120" hidden="true">
+      <c r="A120" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="B120" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="C120" s="2"/>
+      <c r="D120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E120" s="2"/>
+      <c r="F120" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G120" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J120" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K120" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="L120" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="M120" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="N120" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="O120" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="P120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q120" s="2"/>
+      <c r="R120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S120" t="s" s="2">
+        <v>529</v>
+      </c>
+      <c r="T120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF120" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="AG120" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH120" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ120" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL120" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="AM120" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN120" t="s" s="2">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="121" hidden="true">
+      <c r="A121" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="B121" t="s" s="2">
+        <v>446</v>
+      </c>
+      <c r="C121" s="2"/>
+      <c r="D121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E121" s="2"/>
+      <c r="F121" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G121" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K121" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="L121" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="M121" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="N121" s="2"/>
+      <c r="O121" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="P121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q121" s="2"/>
+      <c r="R121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF121" t="s" s="2">
+        <v>446</v>
+      </c>
+      <c r="AG121" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH121" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ121" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL121" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AM121" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN121" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AN111">
+  <autoFilter ref="A1:AN121">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -14664,7 +15842,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI110">
+  <conditionalFormatting sqref="A2:AI120">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>